<commit_message>
ACADIAQPR-14118: Replicate ORE Cross_Currency_Swap_rebalancing in QuantLibXL
Add the XccySwapRebalancing.xlsx example workbook, which rebuilds the USD and EUR curves (FedFunds, EONIA, LIBOR-3M/6M, EURIBOR-3M/6M, EUR-IN-USD) and the resetting EUR/USD cross-currency swap using QuantExt functionality only, matching ORE's NPV exactly and its cashflows to output precision. Extend the wrapped QuantExt rate helpers with the index-given flags and the FX settlement days, FX calendar and telescopic value date parameters needed for the replication, add the 30/360 (USA) day counter, and rename some helper parameters to fit the gensrc length limit.
</commit_message>
<xml_diff>
--- a/QuantLibXL/StandaloneExamples/QuantExt/QuantExtRateHelpers.xlsx
+++ b/QuantLibXL/StandaloneExamples/QuantExt/QuantExtRateHelpers.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eehlers\AppData\Local\Temp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\erik\repos\qla-dx1-ee\QuantLibXL\StandaloneExamples\QuantExt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB427A3F-1BA7-4351-BD21-01F8C156372B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{176D719E-02A0-410F-A861-6ECB51912B84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{CF2B5781-4466-47E6-A71C-B5120BD0E61C}"/>
   </bookViews>
@@ -1694,13 +1694,13 @@
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B18" t="e">
-        <f>_xll.qlBasisTwoSwapHelper("BasisTwoSwapHelper",B5,B6,B7,B8,B9,B10,B11,B12,B13,B14,B15,B16,B17,FALSE,Setup!$C$3:$C$19)</f>
-        <v>#NUM!</v>
+      <c r="B18" t="str">
+        <f>_xll.qlBasisTwoSwapHelper("BasisTwoSwapHelper",B5,B6,B7,B8,B9,B10,B11,B12,B13,B14,B15,B16,B17,TRUE,TRUE,FALSE,Setup!$C$3:$C$19)</f>
+        <v>BasisTwoSwapHelper#0000</v>
       </c>
       <c r="D18" t="str">
-        <f ca="1">_xll.ohRangeRetrieveError(B18)</f>
-        <v>qlBasisTwoSwapHelper - input value is vector or matrix, expected scalar</v>
+        <f>_xll.ohRangeRetrieveError(B18)</f>
+        <v/>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -1928,13 +1928,13 @@
       <c r="A48" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B48" t="e">
-        <f>_xll.qlTenorBasisSwapHelper("TenorBasisSwapHelper",B37,B38,B39,B40,B41,B42,B43,B44,B45,B46,B47,FALSE,Setup!$C$3:$C$19)</f>
-        <v>#NUM!</v>
+      <c r="B48" t="str">
+        <f>_xll.qlTenorBasisSwapHelper("TenorBasisSwapHelper",B37,B38,B39,B40,B41,B42,B43,B44,B45,B46,B47,TRUE,TRUE,FALSE,Setup!$C$3:$C$19)</f>
+        <v>TenorBasisSwapHelper#0000</v>
       </c>
       <c r="D48" t="str">
-        <f ca="1">_xll.ohRangeRetrieveError(B48)</f>
-        <v>qlTenorBasisSwapHelper - input value is vector or matrix, expected scalar</v>
+        <f>_xll.ohRangeRetrieveError(B48)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -2081,13 +2081,13 @@
       <c r="A17" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B17" t="e">
-        <f>_xll.qlCrossCcyBasisSwapHelper("CrossCcyBasisSwapHelper",B5,B6,B7,B8,B9,B10,B11,B12,B13,B14,B15,B16,FALSE,Setup!$C$3:$C$19)</f>
-        <v>#NUM!</v>
+      <c r="B17" t="str">
+        <f>_xll.qlCrossCcyBasisSwapHelper("CrossCcyBasisSwapHelper",B5,B6,B7,B8,B9,B10,B11,B12,B13,B14,B15,B16,2,"NullCalendar",FALSE,FALSE,Setup!$C$3:$C$19)</f>
+        <v>CrossCcyBasisSwapHelper#0000</v>
       </c>
       <c r="D17" t="str">
-        <f ca="1">_xll.ohRangeRetrieveError(B17)</f>
-        <v>qlCrossCcyBasisSwapHelper - input value is vector or matrix, expected scalar</v>
+        <f>_xll.ohRangeRetrieveError(B17)</f>
+        <v/>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
@@ -2208,13 +2208,13 @@
       <c r="A33" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B33" t="e">
-        <f>_xll.qlCrossCcyBasisMtMResetSwapHelper("CrossCcyBasisMtMResetSwapHelper",B21,B22,B23,B24,B25,B26,B27,B28,B29,B30,B31,B32,FALSE,Setup!$C$3:$C$19)</f>
-        <v>#NUM!</v>
+      <c r="B33" t="str">
+        <f>_xll.qlCrossCcyBasisMtMResetSwapHelper("CrossCcyBasisMtMResetSwapHelper",B21,B22,B23,B24,B25,B26,B27,B28,B29,B30,B31,B32,2,"NullCalendar",FALSE,FALSE,Setup!$C$3:$C$19)</f>
+        <v>CrossCcyBasisMtMResetSwapHelper#0000</v>
       </c>
       <c r="D33" t="str">
-        <f ca="1">_xll.ohRangeRetrieveError(B33)</f>
-        <v>qlCrossCcyBasisMtMResetSwapHelper - input value is vector or matrix, expected scalar</v>
+        <f>_xll.ohRangeRetrieveError(B33)</f>
+        <v/>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>